<commit_message>
Migrate to pure Python backend, remove C++ codebase and intermediate JSON files
</commit_message>
<xml_diff>
--- a/data/central payroll/SALARY SHEET 26-27.xlsx
+++ b/data/central payroll/SALARY SHEET 26-27.xlsx
@@ -802,7 +802,7 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>SALARY SHEET — FEBRUARY 2027 (FY 26-27)</t>
+          <t>CENTRAL SALARY REGISTER — FEBRUARY 2027 (FY 26-27)</t>
         </is>
       </c>
     </row>
@@ -1015,7 +1015,7 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>SALARY SHEET — MARCH 2027 (FY 26-27)</t>
+          <t>CENTRAL SALARY REGISTER — MARCH 2027 (FY 26-27)</t>
         </is>
       </c>
     </row>
@@ -1356,16 +1356,16 @@
         <v>20000</v>
       </c>
       <c r="J6" s="5" t="n">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="K6" s="5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L6" s="5" t="n">
         <v>0</v>
       </c>
       <c r="M6" s="5" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="N6" s="5" t="n">
         <v>31</v>
@@ -1377,12 +1377,16 @@
         <v>20000</v>
       </c>
       <c r="Q6" s="7" t="n">
-        <v>0</v>
+        <v>1500</v>
       </c>
       <c r="R6" s="7" t="n">
-        <v>20000</v>
-      </c>
-      <c r="S6" s="6" t="inlineStr"/>
+        <v>18500</v>
+      </c>
+      <c r="S6" s="6" t="inlineStr">
+        <is>
+          <t>Updated via in-process batch</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="3">
@@ -1441,7 +1445,7 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>SALARY SHEET — MAY 2026 (FY 26-27)</t>
+          <t>CENTRAL SALARY REGISTER — MAY 2026 (FY 26-27)</t>
         </is>
       </c>
     </row>
@@ -1709,7 +1713,7 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>SALARY SHEET — JUNE 2026 (FY 26-27)</t>
+          <t>CENTRAL SALARY REGISTER — JUNE 2026 (FY 26-27)</t>
         </is>
       </c>
     </row>
@@ -1977,7 +1981,7 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>SALARY SHEET — JULY 2026 (FY 26-27)</t>
+          <t>CENTRAL SALARY REGISTER — JULY 2026 (FY 26-27)</t>
         </is>
       </c>
     </row>
@@ -2245,7 +2249,7 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>SALARY SHEET — AUGUST 2026 (FY 26-27)</t>
+          <t>CENTRAL SALARY REGISTER — AUGUST 2026 (FY 26-27)</t>
         </is>
       </c>
     </row>
@@ -2513,7 +2517,7 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>SALARY SHEET — SEPTEMBER 2026 (FY 26-27)</t>
+          <t>CENTRAL SALARY REGISTER — SEPTEMBER 2026 (FY 26-27)</t>
         </is>
       </c>
     </row>
@@ -2726,7 +2730,7 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>SALARY SHEET — NOVEMBER 2026 (FY 26-27)</t>
+          <t>CENTRAL SALARY REGISTER — NOVEMBER 2026 (FY 26-27)</t>
         </is>
       </c>
     </row>
@@ -2939,7 +2943,7 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>SALARY SHEET — DECEMBER 2026 (FY 26-27)</t>
+          <t>CENTRAL SALARY REGISTER — DECEMBER 2026 (FY 26-27)</t>
         </is>
       </c>
     </row>
@@ -3152,7 +3156,7 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>SALARY SHEET — JANUARY 2027 (FY 26-27)</t>
+          <t>CENTRAL SALARY REGISTER — JANUARY 2027 (FY 26-27)</t>
         </is>
       </c>
     </row>

</xml_diff>